<commit_message>
Updated Prgram Output KPIs an Service Unit KPIs
</commit_message>
<xml_diff>
--- a/data/Program Output KPIs.xlsx
+++ b/data/Program Output KPIs.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Learning\Miscellaneous\KPIDashboard\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cgiar-my.sharepoint.com/personal/s_lewis_cgiar_org/Documents/TAAT/R4D/KPIS/Alekeh/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14A52755-621F-4A75-A4AB-A318B01555D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="53" documentId="8_{13FACF68-87A9-442A-8EEC-FB2E7358B28E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ACD021D2-0AC7-4431-8F3A-6AAFC4BD0DDC}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7D6C42FC-A6F5-4FB3-BCAA-02C3B0CCB318}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{7D6C42FC-A6F5-4FB3-BCAA-02C3B0CCB318}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -195,13 +195,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="166" formatCode="0.0%"/>
-    <numFmt numFmtId="167" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;??_);_(@_)"/>
+  <numFmts count="3">
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="169" formatCode="0.0"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -490,189 +489,15 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="10" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="4" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="14" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="14" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="4" fillId="3" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="3" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="3" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="3" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="13" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -690,6 +515,156 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="14" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="169" fontId="5" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="3" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="4" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="8" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="14" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="12" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="13" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1027,373 +1002,373 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{436DF3B9-9B26-4648-BD64-23BB8D8864D3}">
-  <dimension ref="A1:H21"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <dimension ref="A1:F21"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10.88671875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="6.5546875" style="36" customWidth="1"/>
-    <col min="3" max="3" width="35.21875" style="46" customWidth="1"/>
-    <col min="4" max="4" width="9.44140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.21875" style="57" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.5546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.90625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="6.54296875" style="19" customWidth="1"/>
+    <col min="3" max="3" width="35.1796875" style="19" customWidth="1"/>
+    <col min="4" max="4" width="9.453125" style="43" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.6328125" style="44" customWidth="1"/>
+    <col min="6" max="6" width="8.54296875" style="45" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" ht="36.6" thickBot="1">
-      <c r="B1" s="28" t="s">
+    <row r="1" spans="1:6" s="1" customFormat="1" ht="36.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B1" s="52" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="37" t="s">
+      <c r="C1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="48" t="s">
+      <c r="E1" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="F1" s="23" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:6" s="3" customFormat="1" ht="28.5" customHeight="1">
-      <c r="A2" s="61" t="s">
+    <row r="2" spans="1:6" s="2" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="29" t="s">
+      <c r="B2" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="38" t="s">
+      <c r="C2" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="11">
+      <c r="D2" s="24">
         <v>272</v>
       </c>
-      <c r="E2" s="49">
-        <v>220</v>
-      </c>
-      <c r="F2" s="12"/>
-    </row>
-    <row r="3" spans="1:6" s="3" customFormat="1" ht="28.5" customHeight="1">
-      <c r="A3" s="62"/>
-      <c r="B3" s="30" t="s">
+      <c r="E2" s="25">
+        <v>217</v>
+      </c>
+      <c r="F2" s="26"/>
+    </row>
+    <row r="3" spans="1:6" s="2" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="4"/>
+      <c r="B3" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="39" t="s">
+      <c r="C3" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="27">
         <v>2</v>
       </c>
-      <c r="E3" s="50">
+      <c r="E3" s="20">
         <v>1.3</v>
       </c>
-      <c r="F3" s="13"/>
-    </row>
-    <row r="4" spans="1:6" s="3" customFormat="1" ht="28.5" customHeight="1" thickBot="1">
-      <c r="A4" s="63"/>
-      <c r="B4" s="31" t="s">
+      <c r="F3" s="28"/>
+    </row>
+    <row r="4" spans="1:6" s="2" customFormat="1" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="5"/>
+      <c r="B4" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="40" t="s">
+      <c r="C4" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="14">
+      <c r="D4" s="29">
         <v>1</v>
       </c>
-      <c r="E4" s="51">
+      <c r="E4" s="30">
         <v>6</v>
       </c>
-      <c r="F4" s="15"/>
-    </row>
-    <row r="5" spans="1:6" s="3" customFormat="1" ht="28.5" customHeight="1">
-      <c r="A5" s="64" t="s">
+      <c r="F4" s="31"/>
+    </row>
+    <row r="5" spans="1:6" s="2" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="32" t="s">
+      <c r="B5" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="41" t="s">
+      <c r="C5" s="50" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="18">
+      <c r="D5" s="32">
         <v>150</v>
       </c>
-      <c r="E5" s="52">
+      <c r="E5" s="33">
         <v>113</v>
       </c>
-      <c r="F5" s="19">
+      <c r="F5" s="14">
         <f>67/113</f>
         <v>0.59292035398230092</v>
       </c>
     </row>
-    <row r="6" spans="1:6" s="3" customFormat="1" ht="28.5" customHeight="1">
-      <c r="A6" s="65"/>
-      <c r="B6" s="33" t="s">
+    <row r="6" spans="1:6" s="2" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="7"/>
+      <c r="B6" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="42" t="s">
+      <c r="C6" s="51" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="16">
+      <c r="D6" s="34">
         <v>60</v>
       </c>
-      <c r="E6" s="53">
+      <c r="E6" s="35">
         <v>103</v>
       </c>
-      <c r="F6" s="20">
+      <c r="F6" s="16">
         <f>50/103</f>
         <v>0.4854368932038835</v>
       </c>
     </row>
-    <row r="7" spans="1:6" s="3" customFormat="1" ht="28.5" customHeight="1">
-      <c r="A7" s="65"/>
-      <c r="B7" s="33" t="s">
+    <row r="7" spans="1:6" s="2" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="7"/>
+      <c r="B7" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="43" t="s">
+      <c r="C7" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="17">
+      <c r="D7" s="36">
         <v>12000</v>
       </c>
-      <c r="E7" s="53">
+      <c r="E7" s="35">
         <v>12612</v>
       </c>
-      <c r="F7" s="20">
+      <c r="F7" s="16">
         <v>0.43909999999999999</v>
       </c>
     </row>
-    <row r="8" spans="1:6" s="3" customFormat="1" ht="36" customHeight="1" thickBot="1">
-      <c r="A8" s="66"/>
-      <c r="B8" s="34" t="s">
+    <row r="8" spans="1:6" s="2" customFormat="1" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="8"/>
+      <c r="B8" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="44" t="s">
+      <c r="C8" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="D8" s="21">
+      <c r="D8" s="37">
         <v>150</v>
       </c>
-      <c r="E8" s="54">
+      <c r="E8" s="38">
         <v>1444</v>
       </c>
-      <c r="F8" s="22">
+      <c r="F8" s="18">
         <v>0.33650000000000002</v>
       </c>
     </row>
-    <row r="9" spans="1:6" s="3" customFormat="1" ht="28.5" customHeight="1">
-      <c r="A9" s="61" t="s">
+    <row r="9" spans="1:6" s="2" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B9" s="35" t="s">
+      <c r="B9" s="53" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="45" t="s">
+      <c r="C9" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="D9" s="23">
+      <c r="D9" s="39">
+        <v>6</v>
+      </c>
+      <c r="E9" s="40">
+        <v>15</v>
+      </c>
+      <c r="F9" s="26"/>
+    </row>
+    <row r="10" spans="1:6" s="2" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="4"/>
+      <c r="B10" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="D10" s="47">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="E10" s="49">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="F10" s="28"/>
+    </row>
+    <row r="11" spans="1:6" s="2" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="4"/>
+      <c r="B11" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="D11" s="46">
         <v>1</v>
       </c>
-      <c r="E9" s="55">
+      <c r="E11" s="48">
+        <v>1</v>
+      </c>
+      <c r="F11" s="28"/>
+    </row>
+    <row r="12" spans="1:6" s="2" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="4"/>
+      <c r="B12" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="D12" s="27">
+        <v>20</v>
+      </c>
+      <c r="E12" s="41">
+        <v>51</v>
+      </c>
+      <c r="F12" s="28"/>
+    </row>
+    <row r="13" spans="1:6" s="2" customFormat="1" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="5"/>
+      <c r="B13" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="D13" s="29">
+        <v>30</v>
+      </c>
+      <c r="E13" s="30">
+        <v>23</v>
+      </c>
+      <c r="F13" s="31"/>
+    </row>
+    <row r="14" spans="1:6" s="2" customFormat="1" ht="36.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="D14" s="27">
+        <v>30</v>
+      </c>
+      <c r="E14" s="41">
+        <v>140</v>
+      </c>
+      <c r="F14" s="42"/>
+    </row>
+    <row r="15" spans="1:6" s="2" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="4"/>
+      <c r="B15" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="D15" s="27">
+        <v>25</v>
+      </c>
+      <c r="E15" s="41">
+        <v>38</v>
+      </c>
+      <c r="F15" s="28"/>
+    </row>
+    <row r="16" spans="1:6" s="2" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A16" s="4"/>
+      <c r="B16" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="D16" s="27">
+        <v>30</v>
+      </c>
+      <c r="E16" s="41">
+        <v>8</v>
+      </c>
+      <c r="F16" s="28"/>
+    </row>
+    <row r="17" spans="1:6" s="2" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A17" s="4"/>
+      <c r="B17" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="D17" s="27">
+        <v>30</v>
+      </c>
+      <c r="E17" s="41">
+        <v>18</v>
+      </c>
+      <c r="F17" s="28"/>
+    </row>
+    <row r="18" spans="1:6" s="2" customFormat="1" ht="36.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="5"/>
+      <c r="B18" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="C18" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="D18" s="29">
         <v>15</v>
       </c>
-      <c r="F9" s="12"/>
-    </row>
-    <row r="10" spans="1:6" s="3" customFormat="1" ht="28.5" customHeight="1">
-      <c r="A10" s="62"/>
-      <c r="B10" s="30" t="s">
-        <v>24</v>
-      </c>
-      <c r="C10" s="43" t="s">
-        <v>25</v>
-      </c>
-      <c r="D10" s="6">
-        <v>1.4999999999999999E-2</v>
-      </c>
-      <c r="E10" s="47">
-        <v>1.4999999999999999E-2</v>
-      </c>
-      <c r="F10" s="13"/>
-    </row>
-    <row r="11" spans="1:6" s="3" customFormat="1" ht="28.5" customHeight="1">
-      <c r="A11" s="62"/>
-      <c r="B11" s="30" t="s">
-        <v>26</v>
-      </c>
-      <c r="C11" s="43" t="s">
-        <v>27</v>
-      </c>
-      <c r="D11" s="8">
-        <v>1</v>
-      </c>
-      <c r="E11" s="56">
-        <v>1</v>
-      </c>
-      <c r="F11" s="13"/>
-    </row>
-    <row r="12" spans="1:6" s="3" customFormat="1" ht="28.5" customHeight="1">
-      <c r="A12" s="62"/>
-      <c r="B12" s="30" t="s">
-        <v>28</v>
-      </c>
-      <c r="C12" s="39" t="s">
-        <v>29</v>
-      </c>
-      <c r="D12" s="2">
-        <v>20</v>
-      </c>
-      <c r="E12" s="56">
-        <v>51</v>
-      </c>
-      <c r="F12" s="13"/>
-    </row>
-    <row r="13" spans="1:6" s="3" customFormat="1" ht="28.5" customHeight="1" thickBot="1">
-      <c r="A13" s="63"/>
-      <c r="B13" s="31" t="s">
+      <c r="E18" s="30">
         <v>30</v>
       </c>
-      <c r="C13" s="40" t="s">
-        <v>31</v>
-      </c>
-      <c r="D13" s="14">
-        <v>30</v>
-      </c>
-      <c r="E13" s="51">
-        <v>19</v>
-      </c>
-      <c r="F13" s="15"/>
-    </row>
-    <row r="14" spans="1:6" s="3" customFormat="1" ht="36" customHeight="1">
-      <c r="A14" s="61" t="s">
-        <v>32</v>
-      </c>
-      <c r="B14" s="29" t="s">
-        <v>33</v>
-      </c>
-      <c r="C14" s="38" t="s">
-        <v>34</v>
-      </c>
-      <c r="D14" s="11">
-        <v>30</v>
-      </c>
-      <c r="E14" s="55">
-        <v>38</v>
-      </c>
-      <c r="F14" s="24"/>
-    </row>
-    <row r="15" spans="1:6" s="3" customFormat="1" ht="12">
-      <c r="A15" s="62"/>
-      <c r="B15" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="C15" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="D15" s="2">
-        <v>30</v>
-      </c>
-      <c r="E15" s="56">
-        <v>83</v>
-      </c>
-      <c r="F15" s="25"/>
-    </row>
-    <row r="16" spans="1:6" s="3" customFormat="1" ht="24">
-      <c r="A16" s="62"/>
-      <c r="B16" s="30" t="s">
-        <v>37</v>
-      </c>
-      <c r="C16" s="39" t="s">
-        <v>38</v>
-      </c>
-      <c r="D16" s="2">
-        <v>30</v>
-      </c>
-      <c r="E16" s="56">
-        <v>8</v>
-      </c>
-      <c r="F16" s="13"/>
-    </row>
-    <row r="17" spans="1:6" s="3" customFormat="1" ht="24">
-      <c r="A17" s="62"/>
-      <c r="B17" s="30" t="s">
-        <v>39</v>
-      </c>
-      <c r="C17" s="39" t="s">
-        <v>40</v>
-      </c>
-      <c r="D17" s="2">
-        <v>30</v>
-      </c>
-      <c r="E17" s="56">
-        <v>18</v>
-      </c>
-      <c r="F17" s="13"/>
-    </row>
-    <row r="18" spans="1:6" s="3" customFormat="1" ht="36.6" thickBot="1">
-      <c r="A18" s="63"/>
-      <c r="B18" s="31" t="s">
-        <v>41</v>
-      </c>
-      <c r="C18" s="44" t="s">
-        <v>42</v>
-      </c>
-      <c r="D18" s="14">
-        <v>30</v>
-      </c>
-      <c r="E18" s="51">
-        <v>12</v>
-      </c>
-      <c r="F18" s="15"/>
-    </row>
-    <row r="19" spans="1:6" s="3" customFormat="1" ht="30.6" customHeight="1">
-      <c r="A19" s="61" t="s">
+      <c r="F18" s="31"/>
+    </row>
+    <row r="19" spans="1:6" s="2" customFormat="1" ht="30.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B19" s="29" t="s">
+      <c r="B19" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="C19" s="38" t="s">
+      <c r="C19" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="D19" s="26">
+      <c r="D19" s="54">
         <v>0.25</v>
       </c>
-      <c r="E19" s="58">
+      <c r="E19" s="55">
         <v>0.41666666666666669</v>
       </c>
-      <c r="F19" s="12"/>
-    </row>
-    <row r="20" spans="1:6" s="3" customFormat="1" ht="24">
-      <c r="A20" s="62"/>
-      <c r="B20" s="30" t="s">
+      <c r="F19" s="26"/>
+    </row>
+    <row r="20" spans="1:6" s="2" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A20" s="4"/>
+      <c r="B20" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="C20" s="39" t="s">
+      <c r="C20" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="D20" s="7">
+      <c r="D20" s="56">
         <v>0.25</v>
       </c>
-      <c r="E20" s="59">
+      <c r="E20" s="48">
         <v>0.3611111111111111</v>
       </c>
-      <c r="F20" s="13"/>
-    </row>
-    <row r="21" spans="1:6" s="3" customFormat="1" ht="24.6" thickBot="1">
-      <c r="A21" s="63"/>
-      <c r="B21" s="31" t="s">
+      <c r="F20" s="28"/>
+    </row>
+    <row r="21" spans="1:6" s="2" customFormat="1" ht="24.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="5"/>
+      <c r="B21" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="C21" s="40" t="s">
+      <c r="C21" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="D21" s="27">
+      <c r="D21" s="57">
         <v>0.25</v>
       </c>
-      <c r="E21" s="60">
+      <c r="E21" s="58">
         <v>0.1111111111111111</v>
       </c>
-      <c r="F21" s="15"/>
+      <c r="F21" s="31"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -1403,249 +1378,7 @@
     <mergeCell ref="A9:A13"/>
     <mergeCell ref="A14:A18"/>
   </mergeCells>
-  <conditionalFormatting sqref="E2">
-    <cfRule type="colorScale" priority="20">
-      <colorScale>
-        <cfvo type="formula" val="$D$2*50%"/>
-        <cfvo type="formula" val="$D$2*75%"/>
-        <cfvo type="formula" val="$D$2"/>
-        <color rgb="FFFF0000"/>
-        <color rgb="FFFFFF00"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E3">
-    <cfRule type="colorScale" priority="19">
-      <colorScale>
-        <cfvo type="formula" val="$D$3*50%"/>
-        <cfvo type="formula" val="$D$3*75%"/>
-        <cfvo type="formula" val="$D$3"/>
-        <color rgb="FFFF0000"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E4">
-    <cfRule type="colorScale" priority="18">
-      <colorScale>
-        <cfvo type="formula" val="$D$4*50%"/>
-        <cfvo type="formula" val="$D$4*75%"/>
-        <cfvo type="formula" val="$D$4"/>
-        <color rgb="FFFF0000"/>
-        <color rgb="FFFFFF00"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E5">
-    <cfRule type="colorScale" priority="17">
-      <colorScale>
-        <cfvo type="formula" val="$D$5*50%"/>
-        <cfvo type="formula" val="$D$5*75%"/>
-        <cfvo type="formula" val="$D$5"/>
-        <color rgb="FFFF0000"/>
-        <color rgb="FFFFFF00"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E6">
-    <cfRule type="colorScale" priority="16">
-      <colorScale>
-        <cfvo type="formula" val="$D$6*50%"/>
-        <cfvo type="formula" val="$D$6*75%"/>
-        <cfvo type="formula" val="$D$6"/>
-        <color rgb="FFFF0000"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E7">
-    <cfRule type="colorScale" priority="15">
-      <colorScale>
-        <cfvo type="formula" val="$D$6*50%"/>
-        <cfvo type="formula" val="$D$7*75%"/>
-        <cfvo type="formula" val="$D$7"/>
-        <color rgb="FFFF0000"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E8">
-    <cfRule type="colorScale" priority="14">
-      <colorScale>
-        <cfvo type="formula" val="$D$8*50%"/>
-        <cfvo type="formula" val="$D$8*75%"/>
-        <cfvo type="formula" val="$D$8"/>
-        <color rgb="FFFF0000"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E9">
-    <cfRule type="colorScale" priority="13">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="formula" val="$D$9"/>
-        <color rgb="FFFF0000"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E10">
-    <cfRule type="colorScale" priority="12">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="formula" val="$D$10"/>
-        <color rgb="FFFF0000"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E11">
-    <cfRule type="colorScale" priority="11">
-      <colorScale>
-        <cfvo type="formula" val="$D$11*50%"/>
-        <cfvo type="formula" val="$D$11*75%"/>
-        <cfvo type="formula" val="$D$11"/>
-        <color rgb="FFFF0000"/>
-        <color rgb="FFFFFF00"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E12">
-    <cfRule type="colorScale" priority="10">
-      <colorScale>
-        <cfvo type="formula" val="$D$12*50%"/>
-        <cfvo type="formula" val="$D$12*75%"/>
-        <cfvo type="formula" val="$D$12"/>
-        <color rgb="FFFF0000"/>
-        <color rgb="FFFFFF00"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E13">
-    <cfRule type="colorScale" priority="9">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="formula" val="$D$13*75%"/>
-        <cfvo type="formula" val="$D$13"/>
-        <color rgb="FFFF0000"/>
-        <color rgb="FFFFFF00"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E14">
-    <cfRule type="colorScale" priority="8">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="formula" val="$D$14*75%"/>
-        <cfvo type="formula" val="$D$14"/>
-        <color rgb="FFFF0000"/>
-        <color rgb="FFFFFF00"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E15">
-    <cfRule type="colorScale" priority="7">
-      <colorScale>
-        <cfvo type="formula" val="$D$15*50%"/>
-        <cfvo type="formula" val="$D$15*75%"/>
-        <cfvo type="formula" val="$D$15"/>
-        <color rgb="FFFF0000"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E16">
-    <cfRule type="colorScale" priority="6">
-      <colorScale>
-        <cfvo type="formula" val="$D$16*50%"/>
-        <cfvo type="formula" val="$D$16*75%"/>
-        <cfvo type="formula" val="$D$16"/>
-        <color rgb="FFFF0000"/>
-        <color rgb="FFFFFF00"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E17">
-    <cfRule type="colorScale" priority="5">
-      <colorScale>
-        <cfvo type="formula" val="$D$17*50%"/>
-        <cfvo type="formula" val="$D$17*75%"/>
-        <cfvo type="formula" val="$D$17"/>
-        <color rgb="FFFF0000"/>
-        <color rgb="FFFFFF00"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E18">
-    <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="formula" val="$D$18*50%"/>
-        <cfvo type="formula" val="$D$18*75%"/>
-        <cfvo type="formula" val="$D$18"/>
-        <color rgb="FFFF0000"/>
-        <color rgb="FFFFFF00"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E19">
-    <cfRule type="colorScale" priority="4">
-      <colorScale>
-        <cfvo type="formula" val="$D$19*50%"/>
-        <cfvo type="formula" val="$D$19*75%"/>
-        <cfvo type="formula" val="$D$19"/>
-        <color rgb="FFFF0000"/>
-        <color rgb="FFFFFF00"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E20">
-    <cfRule type="colorScale" priority="3">
-      <colorScale>
-        <cfvo type="formula" val="$D$20*50%"/>
-        <cfvo type="formula" val="$D$20*75%"/>
-        <cfvo type="formula" val="$D$20"/>
-        <color rgb="FFFF0000"/>
-        <color rgb="FFFFFF00"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E21">
-    <cfRule type="colorScale" priority="2">
-      <colorScale>
-        <cfvo type="formula" val="$D$21*50%"/>
-        <cfvo type="formula" val="$D$21*75%"/>
-        <cfvo type="formula" val="$D$21"/>
-        <color rgb="FFFF0000"/>
-        <color rgb="FFFFFF00"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
-<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
-  <clbl:label id="{9d258917-277f-42cd-a3cd-14c4e9ee58bc}" enabled="1" method="Standard" siteId="{38ae3bcd-9579-4fd4-adda-b42e1495d55a}" contentBits="0" removed="0"/>
-</clbl:labelList>
 </file>
</xml_diff>

<commit_message>
Added updated Program Output KPIs
</commit_message>
<xml_diff>
--- a/data/Program Output KPIs.xlsx
+++ b/data/Program Output KPIs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Learning\Miscellaneous\KPIDashboard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40405010-A0C7-420C-A3B2-6E5CC8B2595A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04601E51-D4E5-40E9-9E5A-B76895A352FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7D6C42FC-A6F5-4FB3-BCAA-02C3B0CCB318}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{7D6C42FC-A6F5-4FB3-BCAA-02C3B0CCB318}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
   <si>
     <t>Annual Target</t>
   </si>
@@ -107,9 +107,6 @@
     <t>KPI 7</t>
   </si>
   <si>
-    <t>Key Performance Indicator (KPI)</t>
-  </si>
-  <si>
     <t>Number of delivery partners trained</t>
   </si>
   <si>
@@ -198,6 +195,12 @@
   </si>
   <si>
     <t>KPI Metric</t>
+  </si>
+  <si>
+    <t>Key Performance Indicator (KPI) Pillar</t>
+  </si>
+  <si>
+    <t>KPI</t>
   </si>
 </sst>
 </file>
@@ -272,7 +275,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="21">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -480,19 +483,6 @@
         <color indexed="64"/>
       </right>
       <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
         <color indexed="64"/>
       </top>
       <bottom style="medium">
@@ -558,7 +548,7 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -657,25 +647,22 @@
     <xf numFmtId="9" fontId="3" fillId="2" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="4" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="5" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="20" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="5" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -684,22 +671,22 @@
     <xf numFmtId="166" fontId="3" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="18" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="18" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="166" fontId="5" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="19" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="17" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="19" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="18" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="20" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1078,23 +1065,25 @@
     <col min="5" max="5" width="9.6640625" style="21" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1" ht="36.6" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="34"/>
-      <c r="B1" s="35" t="s">
-        <v>22</v>
-      </c>
-      <c r="C1" s="35" t="s">
+    <row r="1" spans="1:5" s="1" customFormat="1" ht="48.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="34" t="s">
         <v>52</v>
       </c>
-      <c r="D1" s="36" t="s">
+      <c r="B1" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="C1" s="34" t="s">
+        <v>51</v>
+      </c>
+      <c r="D1" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="37" t="s">
+      <c r="E1" s="36" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="2" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="49" t="s">
+      <c r="A2" s="48" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="22" t="s">
@@ -1106,12 +1095,12 @@
       <c r="D2" s="15">
         <v>272</v>
       </c>
-      <c r="E2" s="38">
+      <c r="E2" s="37">
         <v>217</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="2" customFormat="1" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="50"/>
+      <c r="A3" s="49"/>
       <c r="B3" s="23" t="s">
         <v>16</v>
       </c>
@@ -1121,12 +1110,12 @@
       <c r="D3" s="17">
         <v>2</v>
       </c>
-      <c r="E3" s="39">
+      <c r="E3" s="38">
         <v>1.7</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="2" customFormat="1" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="51"/>
+      <c r="A4" s="50"/>
       <c r="B4" s="24" t="s">
         <v>15</v>
       </c>
@@ -1136,32 +1125,32 @@
       <c r="D4" s="18">
         <v>13</v>
       </c>
-      <c r="E4" s="40">
+      <c r="E4" s="39">
         <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="2" customFormat="1" ht="26.55" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="52" t="s">
+      <c r="A5" s="51" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="55" t="s">
+      <c r="B5" s="54" t="s">
         <v>17</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D5" s="15">
         <v>150</v>
       </c>
-      <c r="E5" s="41">
+      <c r="E5" s="40">
         <v>113</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="2" customFormat="1" ht="24" x14ac:dyDescent="0.25">
-      <c r="A6" s="53"/>
-      <c r="B6" s="56"/>
+      <c r="A6" s="52"/>
+      <c r="B6" s="55"/>
       <c r="C6" s="26" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D6" s="27">
         <v>0.5</v>
@@ -1171,25 +1160,25 @@
       </c>
     </row>
     <row r="7" spans="1:5" s="2" customFormat="1" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="53"/>
-      <c r="B7" s="57" t="s">
+      <c r="A7" s="52"/>
+      <c r="B7" s="56" t="s">
         <v>19</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D7" s="19">
         <v>60</v>
       </c>
-      <c r="E7" s="42">
+      <c r="E7" s="41">
         <v>103</v>
       </c>
     </row>
     <row r="8" spans="1:5" s="2" customFormat="1" ht="24" x14ac:dyDescent="0.25">
-      <c r="A8" s="53"/>
-      <c r="B8" s="57"/>
+      <c r="A8" s="52"/>
+      <c r="B8" s="56"/>
       <c r="C8" s="29" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D8" s="27">
         <v>0.5</v>
@@ -1199,25 +1188,25 @@
       </c>
     </row>
     <row r="9" spans="1:5" s="2" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="53"/>
-      <c r="B9" s="57" t="s">
+      <c r="A9" s="52"/>
+      <c r="B9" s="56" t="s">
         <v>20</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D9" s="20">
         <v>12000</v>
       </c>
-      <c r="E9" s="42">
+      <c r="E9" s="41">
         <v>12612</v>
       </c>
     </row>
     <row r="10" spans="1:5" s="2" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="53"/>
-      <c r="B10" s="57"/>
+      <c r="A10" s="52"/>
+      <c r="B10" s="56"/>
       <c r="C10" s="29" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D10" s="27">
         <v>0.5</v>
@@ -1227,25 +1216,25 @@
       </c>
     </row>
     <row r="11" spans="1:5" s="2" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="53"/>
-      <c r="B11" s="57" t="s">
+      <c r="A11" s="52"/>
+      <c r="B11" s="56" t="s">
         <v>21</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D11" s="20">
         <v>150</v>
       </c>
-      <c r="E11" s="42">
+      <c r="E11" s="41">
         <v>1444</v>
       </c>
     </row>
     <row r="12" spans="1:5" s="2" customFormat="1" ht="24.6" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="54"/>
-      <c r="B12" s="58"/>
+      <c r="A12" s="53"/>
+      <c r="B12" s="57"/>
       <c r="C12" s="31" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D12" s="32">
         <v>0.5</v>
@@ -1255,56 +1244,56 @@
       </c>
     </row>
     <row r="13" spans="1:5" s="2" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="49" t="s">
+      <c r="A13" s="48" t="s">
         <v>5</v>
       </c>
       <c r="B13" s="25" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D13" s="16">
         <v>6</v>
       </c>
-      <c r="E13" s="43">
+      <c r="E13" s="42">
         <v>15</v>
       </c>
     </row>
     <row r="14" spans="1:5" s="2" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="50"/>
+      <c r="A14" s="49"/>
       <c r="B14" s="23" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D14" s="9">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="E14" s="44">
+      <c r="E14" s="43">
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
     <row r="15" spans="1:5" s="2" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="50"/>
+      <c r="A15" s="49"/>
       <c r="B15" s="23" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D15" s="10">
         <v>1</v>
       </c>
-      <c r="E15" s="45">
+      <c r="E15" s="44">
         <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:5" s="2" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="50"/>
+      <c r="A16" s="49"/>
       <c r="B16" s="23" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>6</v>
@@ -1312,46 +1301,46 @@
       <c r="D16" s="17">
         <v>20</v>
       </c>
-      <c r="E16" s="46">
+      <c r="E16" s="45">
         <v>51</v>
       </c>
     </row>
     <row r="17" spans="1:5" s="2" customFormat="1" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="51"/>
+      <c r="A17" s="50"/>
       <c r="B17" s="24" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D17" s="18">
         <v>30</v>
       </c>
-      <c r="E17" s="40">
+      <c r="E17" s="39">
         <v>23</v>
       </c>
     </row>
     <row r="18" spans="1:5" s="2" customFormat="1" ht="36.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="49" t="s">
+      <c r="A18" s="48" t="s">
         <v>7</v>
       </c>
       <c r="B18" s="22" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D18" s="15">
         <v>30</v>
       </c>
-      <c r="E18" s="43">
+      <c r="E18" s="42">
         <v>140</v>
       </c>
     </row>
     <row r="19" spans="1:5" s="2" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="50"/>
+      <c r="A19" s="49"/>
       <c r="B19" s="23" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>8</v>
@@ -1359,61 +1348,61 @@
       <c r="D19" s="17">
         <v>25</v>
       </c>
-      <c r="E19" s="46">
+      <c r="E19" s="45">
         <v>38</v>
       </c>
     </row>
     <row r="20" spans="1:5" s="2" customFormat="1" ht="12" x14ac:dyDescent="0.25">
-      <c r="A20" s="50"/>
+      <c r="A20" s="49"/>
       <c r="B20" s="23" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D20" s="17">
         <v>30</v>
       </c>
-      <c r="E20" s="46">
+      <c r="E20" s="45">
         <v>8</v>
       </c>
     </row>
     <row r="21" spans="1:5" s="2" customFormat="1" ht="24" x14ac:dyDescent="0.25">
-      <c r="A21" s="50"/>
+      <c r="A21" s="49"/>
       <c r="B21" s="23" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D21" s="17">
         <v>30</v>
       </c>
-      <c r="E21" s="46">
+      <c r="E21" s="45">
         <v>18</v>
       </c>
     </row>
     <row r="22" spans="1:5" s="2" customFormat="1" ht="24.6" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="51"/>
+      <c r="A22" s="50"/>
       <c r="B22" s="24" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D22" s="18">
         <v>15</v>
       </c>
-      <c r="E22" s="40">
+      <c r="E22" s="39">
         <v>30</v>
       </c>
     </row>
     <row r="23" spans="1:5" s="2" customFormat="1" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="49" t="s">
+      <c r="A23" s="48" t="s">
         <v>9</v>
       </c>
       <c r="B23" s="22" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>10</v>
@@ -1421,14 +1410,14 @@
       <c r="D23" s="11">
         <v>0.25</v>
       </c>
-      <c r="E23" s="47">
+      <c r="E23" s="46">
         <v>0.41666666666666669</v>
       </c>
     </row>
     <row r="24" spans="1:5" s="2" customFormat="1" ht="24" x14ac:dyDescent="0.25">
-      <c r="A24" s="50"/>
+      <c r="A24" s="49"/>
       <c r="B24" s="23" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>11</v>
@@ -1436,14 +1425,14 @@
       <c r="D24" s="12">
         <v>0.25</v>
       </c>
-      <c r="E24" s="45">
+      <c r="E24" s="44">
         <v>0.3611111111111111</v>
       </c>
     </row>
     <row r="25" spans="1:5" s="2" customFormat="1" ht="24.6" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="51"/>
+      <c r="A25" s="50"/>
       <c r="B25" s="24" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C25" s="5" t="s">
         <v>12</v>
@@ -1451,21 +1440,21 @@
       <c r="D25" s="13">
         <v>0.25</v>
       </c>
-      <c r="E25" s="48">
+      <c r="E25" s="47">
         <v>0.1111111111111111</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="9">
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="B11:B12"/>
     <mergeCell ref="A23:A25"/>
     <mergeCell ref="A2:A4"/>
     <mergeCell ref="A5:A12"/>
     <mergeCell ref="A13:A17"/>
     <mergeCell ref="A18:A22"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="B11:B12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
reverted back the files
</commit_message>
<xml_diff>
--- a/data/Program Output KPIs.xlsx
+++ b/data/Program Output KPIs.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cgiar-my.sharepoint.com/personal/s_lewis_cgiar_org/Documents/TAAT/R4D/KPIS/Alekeh/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Learning\Miscellaneous\KPIDashboard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="292" documentId="8_{13FACF68-87A9-442A-8EEC-FB2E7358B28E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4D76AFC2-8B74-457B-8181-12AD3B217C64}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6968D59-EBC4-4AED-9605-DD931C9AF111}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{7D6C42FC-A6F5-4FB3-BCAA-02C3B0CCB318}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{7D6C42FC-A6F5-4FB3-BCAA-02C3B0CCB318}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="59">
   <si>
     <t>Annual Target</t>
   </si>
@@ -107,9 +107,6 @@
     <t>KPI 7</t>
   </si>
   <si>
-    <t>Key Performance Indicator (KPI)</t>
-  </si>
-  <si>
     <t>Number of delivery partners trained</t>
   </si>
   <si>
@@ -198,6 +195,27 @@
   </si>
   <si>
     <t>KPI Metric</t>
+  </si>
+  <si>
+    <t>Key Performance Indicator (KPI) Pillar</t>
+  </si>
+  <si>
+    <t>KPI</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 2026 Actual value </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 2027 Actual value </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 2028 Actual value </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 2029 Actual value </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 2030 Actual value </t>
   </si>
 </sst>
 </file>
@@ -205,10 +223,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
-    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="164" formatCode="0.0%"/>
-    <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="166" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="167" formatCode="#,##0.0"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
@@ -273,7 +291,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="30">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -489,19 +507,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right style="medium">
         <color indexed="64"/>
@@ -542,127 +547,6 @@
     </border>
     <border>
       <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
       <right style="medium">
         <color indexed="64"/>
       </right>
@@ -677,10 +561,10 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -698,10 +582,13 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -719,25 +606,25 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -758,9 +645,15 @@
     <xf numFmtId="9" fontId="5" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="9" fontId="5" fillId="2" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="9" fontId="3" fillId="2" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -770,46 +663,49 @@
     <xf numFmtId="9" fontId="3" fillId="2" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="20" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="19" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="18" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="18" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="17" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="19" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -840,51 +736,6 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="23" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="24" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1223,390 +1074,407 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{436DF3B9-9B26-4648-BD64-23BB8D8864D3}">
-  <dimension ref="A1:E25"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:J25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.90625" style="13" customWidth="1"/>
-    <col min="2" max="2" width="12.1796875" style="7" customWidth="1"/>
-    <col min="3" max="3" width="36.26953125" style="7" customWidth="1"/>
-    <col min="4" max="4" width="9.453125" style="20" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.6328125" style="20" customWidth="1"/>
+    <col min="1" max="1" width="10.88671875" style="14" customWidth="1"/>
+    <col min="2" max="2" width="12.21875" style="8" customWidth="1"/>
+    <col min="3" max="3" width="36.21875" style="8" customWidth="1"/>
+    <col min="4" max="4" width="9.44140625" style="21" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.6640625" style="21" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1" ht="36.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="31"/>
-      <c r="B1" s="32" t="s">
-        <v>22</v>
-      </c>
-      <c r="C1" s="32" t="s">
+    <row r="1" spans="1:10" s="1" customFormat="1" ht="48.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="34" t="s">
         <v>52</v>
       </c>
-      <c r="D1" s="33" t="s">
+      <c r="B1" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="C1" s="34" t="s">
+        <v>51</v>
+      </c>
+      <c r="D1" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="34" t="s">
+      <c r="E1" s="36" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" s="2" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="45" t="s">
+      <c r="F1" s="47" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1" s="47" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1" s="47" t="s">
+        <v>56</v>
+      </c>
+      <c r="I1" s="47" t="s">
+        <v>57</v>
+      </c>
+      <c r="J1" s="47" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" s="2" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="49" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="22" t="s">
         <v>14</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="14">
+      <c r="D2" s="15">
         <v>272</v>
       </c>
-      <c r="E2" s="35">
+      <c r="E2" s="37">
         <v>217</v>
       </c>
     </row>
-    <row r="3" spans="1:5" s="2" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="46"/>
-      <c r="B3" s="22" t="s">
+    <row r="3" spans="1:10" s="2" customFormat="1" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="50"/>
+      <c r="B3" s="23" t="s">
         <v>16</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="42">
+      <c r="D3" s="48">
         <v>2</v>
       </c>
-      <c r="E3" s="43">
+      <c r="E3" s="48">
         <v>1.7</v>
       </c>
     </row>
-    <row r="4" spans="1:5" s="2" customFormat="1" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="47"/>
-      <c r="B4" s="23" t="s">
+    <row r="4" spans="1:10" s="2" customFormat="1" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="51"/>
+      <c r="B4" s="24" t="s">
         <v>15</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="D4" s="44">
+      <c r="D4" s="18">
         <v>13</v>
       </c>
-      <c r="E4" s="36">
+      <c r="E4" s="38">
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:5" s="2" customFormat="1" ht="26.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="48" t="s">
+    <row r="5" spans="1:10" s="2" customFormat="1" ht="26.55" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="52" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="51" t="s">
+      <c r="B5" s="55" t="s">
         <v>17</v>
       </c>
       <c r="C5" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D5" s="15">
+        <v>150</v>
+      </c>
+      <c r="E5" s="39">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" s="2" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A6" s="53"/>
+      <c r="B6" s="56"/>
+      <c r="C6" s="26" t="s">
         <v>47</v>
       </c>
-      <c r="D5" s="14">
+      <c r="D6" s="27">
+        <v>0.5</v>
+      </c>
+      <c r="E6" s="28">
+        <v>0.59</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" s="2" customFormat="1" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="53"/>
+      <c r="B7" s="57" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D7" s="19">
+        <v>60</v>
+      </c>
+      <c r="E7" s="40">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" s="2" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A8" s="53"/>
+      <c r="B8" s="57"/>
+      <c r="C8" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="D8" s="27">
+        <v>0.5</v>
+      </c>
+      <c r="E8" s="30">
+        <v>0.49</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" s="2" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="53"/>
+      <c r="B9" s="57" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D9" s="20">
+        <v>12000</v>
+      </c>
+      <c r="E9" s="40">
+        <v>12612</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" s="2" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="53"/>
+      <c r="B10" s="57"/>
+      <c r="C10" s="29" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" s="27">
+        <v>0.5</v>
+      </c>
+      <c r="E10" s="30">
+        <v>0.44</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" s="2" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="53"/>
+      <c r="B11" s="57" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="D11" s="20">
         <v>150</v>
       </c>
-      <c r="E5" s="56">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" s="2" customFormat="1" ht="24" x14ac:dyDescent="0.25">
-      <c r="A6" s="49"/>
-      <c r="B6" s="52"/>
-      <c r="C6" s="25" t="s">
-        <v>48</v>
-      </c>
-      <c r="D6" s="26">
+      <c r="E11" s="40">
+        <v>1444</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" s="2" customFormat="1" ht="24.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="54"/>
+      <c r="B12" s="58"/>
+      <c r="C12" s="31" t="s">
+        <v>50</v>
+      </c>
+      <c r="D12" s="32">
         <v>0.5</v>
       </c>
-      <c r="E6" s="11">
-        <v>0.59</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" s="2" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="49"/>
-      <c r="B7" s="53" t="s">
-        <v>19</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="D7" s="18">
-        <v>60</v>
-      </c>
-      <c r="E7" s="37">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" s="2" customFormat="1" ht="24" x14ac:dyDescent="0.25">
-      <c r="A8" s="49"/>
-      <c r="B8" s="53"/>
-      <c r="C8" s="27" t="s">
-        <v>46</v>
-      </c>
-      <c r="D8" s="26">
-        <v>0.5</v>
-      </c>
-      <c r="E8" s="55">
-        <v>0.49</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" s="2" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="49"/>
-      <c r="B9" s="53" t="s">
-        <v>20</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="D9" s="19">
-        <v>12000</v>
-      </c>
-      <c r="E9" s="37">
-        <v>12612</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" s="2" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="49"/>
-      <c r="B10" s="53"/>
-      <c r="C10" s="27" t="s">
+      <c r="E12" s="33">
+        <v>0.34</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" s="2" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="49" t="s">
+        <v>5</v>
+      </c>
+      <c r="B13" s="25" t="s">
+        <v>30</v>
+      </c>
+      <c r="C13" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="D10" s="26">
-        <v>0.5</v>
-      </c>
-      <c r="E10" s="55">
-        <v>0.44</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" s="2" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="49"/>
-      <c r="B11" s="53" t="s">
-        <v>21</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="D11" s="19">
-        <v>150</v>
-      </c>
-      <c r="E11" s="37">
-        <v>1444</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" s="2" customFormat="1" ht="24.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="50"/>
-      <c r="B12" s="54"/>
-      <c r="C12" s="28" t="s">
-        <v>51</v>
-      </c>
-      <c r="D12" s="29">
-        <v>0.5</v>
-      </c>
-      <c r="E12" s="30">
-        <v>0.34</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" s="2" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="45" t="s">
-        <v>5</v>
-      </c>
-      <c r="B13" s="24" t="s">
-        <v>31</v>
-      </c>
-      <c r="C13" s="3" t="s">
+      <c r="D13" s="16">
+        <v>6</v>
+      </c>
+      <c r="E13" s="41">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" s="2" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="50"/>
+      <c r="B14" s="23" t="s">
+        <v>33</v>
+      </c>
+      <c r="C14" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="D13" s="15">
-        <v>6</v>
-      </c>
-      <c r="E13" s="38">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" s="2" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="46"/>
-      <c r="B14" s="22" t="s">
+      <c r="D14" s="9">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="E14" s="42">
+        <v>1.4999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" s="2" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="50"/>
+      <c r="B15" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C15" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="D14" s="8">
-        <v>1.4999999999999999E-2</v>
-      </c>
-      <c r="E14" s="39">
-        <v>1.4999999999999999E-2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" s="2" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="46"/>
-      <c r="B15" s="22" t="s">
+      <c r="D15" s="10">
+        <v>1</v>
+      </c>
+      <c r="E15" s="43">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" s="2" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="50"/>
+      <c r="B16" s="23" t="s">
         <v>35</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D15" s="9">
-        <v>1</v>
-      </c>
-      <c r="E15" s="40">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" s="2" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="46"/>
-      <c r="B16" s="22" t="s">
-        <v>36</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D16" s="16">
+      <c r="D16" s="17">
         <v>20</v>
       </c>
-      <c r="E16" s="41">
+      <c r="E16" s="44">
         <v>51</v>
       </c>
     </row>
     <row r="17" spans="1:5" s="2" customFormat="1" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="47"/>
-      <c r="B17" s="23" t="s">
+      <c r="A17" s="51"/>
+      <c r="B17" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D17" s="18">
+        <v>30</v>
+      </c>
+      <c r="E17" s="38">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" s="2" customFormat="1" ht="36.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="49" t="s">
+        <v>7</v>
+      </c>
+      <c r="B18" s="22" t="s">
         <v>37</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="C18" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D17" s="17">
+      <c r="D18" s="15">
         <v>30</v>
       </c>
-      <c r="E17" s="36">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" s="2" customFormat="1" ht="36.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="45" t="s">
-        <v>7</v>
-      </c>
-      <c r="B18" s="21" t="s">
+      <c r="E18" s="41">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" s="2" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="50"/>
+      <c r="B19" s="23" t="s">
         <v>38</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="D18" s="14">
-        <v>30</v>
-      </c>
-      <c r="E18" s="38">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" s="2" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="46"/>
-      <c r="B19" s="22" t="s">
-        <v>39</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D19" s="16">
+      <c r="D19" s="17">
         <v>25</v>
       </c>
-      <c r="E19" s="41">
+      <c r="E19" s="44">
         <v>38</v>
       </c>
     </row>
     <row r="20" spans="1:5" s="2" customFormat="1" ht="12" x14ac:dyDescent="0.25">
-      <c r="A20" s="46"/>
-      <c r="B20" s="22" t="s">
+      <c r="A20" s="50"/>
+      <c r="B20" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D20" s="17">
+        <v>30</v>
+      </c>
+      <c r="E20" s="44">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" s="2" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A21" s="50"/>
+      <c r="B21" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="C21" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D21" s="17">
         <v>30</v>
       </c>
-      <c r="D20" s="16">
+      <c r="E21" s="44">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" s="2" customFormat="1" ht="24.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="51"/>
+      <c r="B22" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="D22" s="18">
+        <v>15</v>
+      </c>
+      <c r="E22" s="38">
         <v>30</v>
       </c>
-      <c r="E20" s="41">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" s="2" customFormat="1" ht="12" x14ac:dyDescent="0.25">
-      <c r="A21" s="46"/>
-      <c r="B21" s="22" t="s">
-        <v>41</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="D21" s="16">
-        <v>30</v>
-      </c>
-      <c r="E21" s="41">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" s="2" customFormat="1" ht="24.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="46"/>
-      <c r="B22" s="57" t="s">
+    </row>
+    <row r="23" spans="1:5" s="2" customFormat="1" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="49" t="s">
+        <v>9</v>
+      </c>
+      <c r="B23" s="22" t="s">
         <v>42</v>
-      </c>
-      <c r="C22" s="58" t="s">
-        <v>33</v>
-      </c>
-      <c r="D22" s="59">
-        <v>15</v>
-      </c>
-      <c r="E22" s="60">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" s="2" customFormat="1" ht="30.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="67" t="s">
-        <v>9</v>
-      </c>
-      <c r="B23" s="64" t="s">
-        <v>43</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D23" s="10">
+      <c r="D23" s="11">
         <v>0.25</v>
       </c>
-      <c r="E23" s="61">
-        <v>0.41666666666666669</v>
+      <c r="E23" s="45">
+        <v>0.41660000000000003</v>
       </c>
     </row>
     <row r="24" spans="1:5" s="2" customFormat="1" ht="24" x14ac:dyDescent="0.25">
-      <c r="A24" s="68"/>
-      <c r="B24" s="65" t="s">
-        <v>44</v>
+      <c r="A24" s="50"/>
+      <c r="B24" s="23" t="s">
+        <v>43</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D24" s="11">
+      <c r="D24" s="12">
         <v>0.25</v>
       </c>
-      <c r="E24" s="62">
+      <c r="E24" s="43">
         <v>0.36</v>
       </c>
     </row>
-    <row r="25" spans="1:5" s="2" customFormat="1" ht="24.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="69"/>
-      <c r="B25" s="66" t="s">
-        <v>45</v>
+    <row r="25" spans="1:5" s="2" customFormat="1" ht="24.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="51"/>
+      <c r="B25" s="24" t="s">
+        <v>44</v>
       </c>
       <c r="C25" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D25" s="12">
+      <c r="D25" s="13">
         <v>0.25</v>
       </c>
-      <c r="E25" s="63">
+      <c r="E25" s="46">
         <v>0.11</v>
       </c>
     </row>
@@ -1622,235 +1490,13 @@
     <mergeCell ref="A13:A17"/>
     <mergeCell ref="A18:A22"/>
   </mergeCells>
-  <conditionalFormatting sqref="E2">
-    <cfRule type="colorScale" priority="21">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="$D$2/2"/>
-        <cfvo type="formula" val="$D$2"/>
-        <color rgb="FFFF0000"/>
-        <color rgb="FFFFFF00"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E3">
-    <cfRule type="colorScale" priority="20">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="formula" val="$D$3/2"/>
-        <cfvo type="formula" val="$D$3"/>
-        <color rgb="FFFF0000"/>
-        <color rgb="FFFFFF00"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E4">
-    <cfRule type="colorScale" priority="19">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="formula" val="$D$4/2"/>
-        <cfvo type="formula" val="$D$4"/>
-        <color rgb="FFFF0000"/>
-        <color rgb="FFFFFF00"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E6">
-    <cfRule type="colorScale" priority="18">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="formula" val="$D$6/2"/>
-        <cfvo type="formula" val="$D$6"/>
-        <color rgb="FFFF0000"/>
-        <color rgb="FFFFFF00"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E7:E8">
-    <cfRule type="colorScale" priority="17">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="formula" val="$D$8/2"/>
-        <cfvo type="formula" val="$D$8"/>
-        <color rgb="FFFF0000"/>
-        <color rgb="FFFFFF00"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E9:E10">
-    <cfRule type="colorScale" priority="16">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="formula" val="$D$10/2"/>
-        <cfvo type="formula" val="$D$10"/>
-        <color rgb="FFFF0000"/>
-        <color rgb="FFFFFF00"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E11">
-    <cfRule type="colorScale" priority="15">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="formula" val="$D$11/2"/>
-        <cfvo type="formula" val="$D$11"/>
-        <color rgb="FFFF0000"/>
-        <color rgb="FFFFFF00"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E13">
-    <cfRule type="colorScale" priority="14">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="$D$13/2"/>
-        <cfvo type="formula" val="$D$13"/>
-        <color rgb="FFFF0000"/>
-        <color rgb="FFFFFF00"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E12">
-    <cfRule type="colorScale" priority="13">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="formula" val="$D$12/2"/>
-        <cfvo type="formula" val="$D$12"/>
-        <color rgb="FFFF0000"/>
-        <color rgb="FFFFFF00"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E14">
-    <cfRule type="colorScale" priority="12">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="formula" val="$D$14/2"/>
-        <cfvo type="formula" val="$D$14"/>
-        <color rgb="FFFF0000"/>
-        <color rgb="FFFFFF00"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E15">
-    <cfRule type="colorScale" priority="11">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="$D$15/2"/>
-        <cfvo type="formula" val="$D$15"/>
-        <color rgb="FFFF0000"/>
-        <color rgb="FFFFFF00"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E16">
-    <cfRule type="colorScale" priority="10">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="formula" val="$D$16/2"/>
-        <cfvo type="formula" val="$D$16"/>
-        <color rgb="FFFF0000"/>
-        <color rgb="FFFFFF00"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E17">
-    <cfRule type="colorScale" priority="9">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="formula" val="$D$17/2"/>
-        <cfvo type="formula" val="$D$17"/>
-        <color rgb="FFFF0000"/>
-        <color rgb="FFFFFF00"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E18">
-    <cfRule type="colorScale" priority="8">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="formula" val="$D$18/2"/>
-        <cfvo type="formula" val="$D$18"/>
-        <color rgb="FFFF0000"/>
-        <color rgb="FFFFFF00"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E19">
-    <cfRule type="colorScale" priority="7">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="formula" val="$D$19/2"/>
-        <cfvo type="formula" val="$D$19"/>
-        <color rgb="FFFF0000"/>
-        <color rgb="FFFFFF00"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E20">
-    <cfRule type="colorScale" priority="5">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="formula" val="$D$20/2"/>
-        <cfvo type="formula" val="$D$20"/>
-        <color rgb="FFFF0000"/>
-        <color rgb="FFFFFF00"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E21">
-    <cfRule type="colorScale" priority="4">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="formula" val="$D$21/2"/>
-        <cfvo type="formula" val="$D$21"/>
-        <color rgb="FFFF0000"/>
-        <color rgb="FFFFFF00"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E22">
-    <cfRule type="colorScale" priority="3">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="formula" val="$D$22/2"/>
-        <cfvo type="formula" val="$D$22"/>
-        <color rgb="FFFF0000"/>
-        <color rgb="FFFFFF00"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E23:E25">
-    <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="formula" val="$D$24/2"/>
-        <cfvo type="formula" val="$D$24"/>
-        <color rgb="FFFF0000"/>
-        <color rgb="FFFFFF00"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{9d258917-277f-42cd-a3cd-14c4e9ee58bc}" enabled="1" method="Standard" siteId="{38ae3bcd-9579-4fd4-adda-b42e1495d55a}" contentBits="0" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>